<commit_message>
fix: refine compartment annotation for vacuole related
</commit_message>
<xml_diff>
--- a/data/organelle_interaction_data.xlsx
+++ b/data/organelle_interaction_data.xlsx
@@ -807,10 +807,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.02123677847022314</v>
+        <v>0.000153003532671201</v>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25">
@@ -1191,10 +1191,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.009793210077770991</v>
+        <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">

</xml_diff>